<commit_message>
Preserve master tank corrections when integrating refreshed vehicles
Move the existing dry-mass and MJ-to-kWh corrections into the retained legacy component workbook, preserving the other 24 recipes and the reviewed car/truck workbooks. Verify the companion hash and invalidate supplementary inventory caches when any of the three vehicle workbooks changes.

Integration retains all 31 vehicle campaign commits, the standalone PV plot, and existing master metals/climate fixes; TRAILS temporal functionality is excluded. Validation: 644 focused tests passed, 1 skipped; strict Sphinx HTML build passed. Full scenario LCIA and score regression references were not rerun or changed.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-truck-legacy-components.xlsx
+++ b/premise/data/additional_inventories/lci-truck-legacy-components.xlsx
@@ -428,6 +428,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1198,7 +1199,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retained legacy truck component, ecoinvent 3.7 import basis; not regenerated by the current vehicle model. </t>
+          <t>Retained legacy truck component; preserves the master-branch dry-mass and electricity correction. Dry-mass correction, 2026-10-10. Evangelisti et al. (2017), doi:10.1016/j.jclepro.2016.11.159, supplementary Hydrogen tank (Scenario S16). Supplement: https://ars.els-cdn.com/content/image/1-s2.0-S0959652616320212-mmc1.docx. SHA256: ca9470c504f61ef58e2e5cc3cad8c06d6cecf17073074ac2ce19dca3678ac49d. Normalize all listed material and processing quantities by 87.71 kg of listed dry materials, not the legacy 119 kg denominator. The main text, scenario labels and supplementary output masses are inconsistent. The difference between nominal output and listed material mass is approximately stored hydrogen, but this interpretation is not explicit in the paper. Dry mass is an explicit modelling boundary, not an assumed missing material. Processing services do not add material mass. Preserve published material ratios and existing supplier proxies, including AlLi for aluminium; these are not validated as current vehicle specifications. Electricity is published in MJ: divide by 3.6 to obtain kWh.</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1233,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>a carbon fiber-resin (CF) composite-wrapped single tank system, with a high density polyethylene (HDPE) liner (i.e., Type IV tanks) capable of storing 5.6 kg usable hydrogen, weighting 119 kg per unit.</t>
+          <t>700-bar hydrogen tank with HDPE (Type IV) liner. Reference output: 1 kg dry tank assembly including tank balance of plant, excluding stored hydrogen. Source listed dry materials total 87.71 kg per assembly.</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1245,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>{"schema version": 1, "role": "retained legacy component", "original workbook": "lci-trucks.xlsx", "original workbook sha256": "0b39c6311dc71dd13254a62901260e23747205cdd4f8871f952c1e77f4128fba", "source database version": "3.7", "model generation version": "not recorded in original workbook", "boundary": "Retained for compatibility with other supplementary inventories; not regenerated by the current carculator_truck model.", "metadata updated": "2026-10-14"}</t>
+          <t>{"schema version": 1, "role": "retained legacy component", "original workbook": "lci-trucks.xlsx", "original workbook sha256": "0b39c6311dc71dd13254a62901260e23747205cdd4f8871f952c1e77f4128fba", "source database version": "3.7", "model generation version": "not recorded in original workbook", "boundary": "Retained for compatibility on the ecoinvent 3.7 import basis; preserves the 2026-10-10 dry-mass and manufacturing-energy correction. Not regenerated by carculator_truck.", "metadata updated": "2026-10-14", "correction source revision": "ff79a88d0e7fc85f116cbe8387a458ac824e94b6", "corrected source workbook sha256": "e4a4b581c35c08e5a9f18a37cdd7bf6306172fd68234c43390bffc0779a7e3ca"}</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1317,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.108151261</v>
+        <v>0.04075932048797173</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1336,6 +1337,11 @@
       <c r="G53" t="inlineStr">
         <is>
           <t>electricity, low voltage</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>12.87 MJ / 3.6 MJ/kWh / 87.71 kg dry assembly = 0.040759320488 kWh/kg. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1352,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.089411765</v>
+        <v>0.1213088587390263</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1366,6 +1372,11 @@
       <c r="G54" t="inlineStr">
         <is>
           <t>metal working, average for chromium steel product manufacturing</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>(10.64) kg / 87.71 kg dry assembly = 0.121308858739 kg/kg. Processing service; excluded from material mass balance. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1387,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.086218487</v>
+        <v>0.1169763994983468</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1396,6 +1407,11 @@
       <c r="G55" t="inlineStr">
         <is>
           <t>polyethylene, high density, granulate</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>(10.26) kg / 87.71 kg dry assembly = 0.116976399498 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1422,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.089411765</v>
+        <v>0.1213088587390263</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1426,6 +1442,11 @@
       <c r="G56" t="inlineStr">
         <is>
           <t>steel, chromium steel 18/8</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>(10.64) kg / 87.71 kg dry assembly = 0.121308858739 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1457,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.249327731</v>
+        <v>0.3382738570288451</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1456,6 +1477,11 @@
       <c r="G57" t="inlineStr">
         <is>
           <t>epoxy resin, liquid</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>(29.67) kg / 87.71 kg dry assembly = 0.338273857029 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1492,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.166218487</v>
+        <v>0.2255159046858967</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1486,6 +1512,11 @@
       <c r="G58" t="inlineStr">
         <is>
           <t>carbon fiber, weaved</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>(19.78) kg / 87.71 kg dry assembly = 0.225515904686 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1527,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.059579832</v>
+        <v>0.08083456846425721</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1516,6 +1547,11 @@
       <c r="G59" t="inlineStr">
         <is>
           <t>aluminium alloy, AlLi</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>(7.09) kg / 87.71 kg dry assembly = 0.0808345684643 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1562,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.047058824</v>
+        <v>0.06384676775738228</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1546,6 +1582,11 @@
       <c r="G60" t="inlineStr">
         <is>
           <t>glass fibre</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>(5.6) kg / 87.71 kg dry assembly = 0.0638467677574 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1627,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.039243697</v>
+        <v>0.05324364382624559</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1606,6 +1647,11 @@
       <c r="G62" t="inlineStr">
         <is>
           <t>polyurethane, flexible foam</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>(4.67) kg / 87.71 kg dry assembly = 0.0532436438262 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1712,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retained legacy truck component, ecoinvent 3.7 import basis; not regenerated by the current vehicle model. </t>
+          <t>Retained legacy truck component; preserves the master-branch dry-mass and electricity correction. Dry-mass correction, 2026-10-10. Evangelisti et al. (2017), doi:10.1016/j.jclepro.2016.11.159, supplementary Hydrogen tank (Scenario S17). Supplement: https://ars.els-cdn.com/content/image/1-s2.0-S0959652616320212-mmc1.docx. SHA256: ca9470c504f61ef58e2e5cc3cad8c06d6cecf17073074ac2ce19dca3678ac49d. Normalize all listed material and processing quantities by 113.169 kg of listed dry materials, not the legacy 93 kg denominator. The main text, scenario labels and supplementary output masses are inconsistent. The difference between nominal output and listed material mass is approximately stored hydrogen, but this interpretation is not explicit in the paper. Dry mass is an explicit modelling boundary, not an assumed missing material. Processing services do not add material mass. Preserve published material ratios and existing supplier proxies, including AlLi for aluminium; these are not validated as current vehicle specifications. Electricity is published in MJ: divide by 3.6 to obtain kWh.</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1746,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>An aluminium lined hydrogen tank (Type III), weighting 93 kg per unit.</t>
+          <t>700-bar hydrogen tank with aluminium (Type III) liner. Reference output: 1 kg dry tank assembly including tank balance of plant, excluding stored hydrogen. Source listed dry materials total 113.169 kg per assembly.</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1758,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>{"schema version": 1, "role": "retained legacy component", "original workbook": "lci-trucks.xlsx", "original workbook sha256": "0b39c6311dc71dd13254a62901260e23747205cdd4f8871f952c1e77f4128fba", "source database version": "3.7", "model generation version": "not recorded in original workbook", "boundary": "Retained for compatibility with other supplementary inventories; not regenerated by the current carculator_truck model.", "metadata updated": "2026-10-14"}</t>
+          <t>{"schema version": 1, "role": "retained legacy component", "original workbook": "lci-trucks.xlsx", "original workbook sha256": "0b39c6311dc71dd13254a62901260e23747205cdd4f8871f952c1e77f4128fba", "source database version": "3.7", "model generation version": "not recorded in original workbook", "boundary": "Retained for compatibility on the ecoinvent 3.7 import basis; preserves the 2026-10-10 dry-mass and manufacturing-energy correction. Not regenerated by carculator_truck.", "metadata updated": "2026-10-14", "correction source revision": "ff79a88d0e7fc85f116cbe8387a458ac824e94b6", "corrected source workbook sha256": "e4a4b581c35c08e5a9f18a37cdd7bf6306172fd68234c43390bffc0779a7e3ca"}</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1830,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.176580645</v>
+        <v>0.04030844724851034</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -1804,6 +1850,11 @@
       <c r="G76" t="inlineStr">
         <is>
           <t>electricity, low voltage</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>16.422 MJ / 3.6 MJ/kWh / 113.169 kg dry assembly = 0.0403084472485 kWh/kg. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1865,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.11388172</v>
+        <v>0.0935856992639327</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -1834,6 +1885,11 @@
       <c r="G77" t="inlineStr">
         <is>
           <t>metal working, average for chromium steel product manufacturing</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>(10.591) kg / 113.169 kg dry assembly = 0.0935856992639 kg/kg. Processing service; excluded from material mass balance. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1900,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.11388172</v>
+        <v>0.0935856992639327</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -1864,6 +1920,11 @@
       <c r="G78" t="inlineStr">
         <is>
           <t>steel, chromium steel 18/8</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>(10.591) kg / 113.169 kg dry assembly = 0.0935856992639 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1935,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.319892473</v>
+        <v>0.2628811777076762</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -1894,6 +1955,11 @@
       <c r="G79" t="inlineStr">
         <is>
           <t>epoxy resin, liquid</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>(29.75) kg / 113.169 kg dry assembly = 0.262881177708 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1970,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.213688172</v>
+        <v>0.1756046267087277</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -1924,6 +1990,11 @@
       <c r="G80" t="inlineStr">
         <is>
           <t>carbon fiber, weaved</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>(19.873) kg / 113.169 kg dry assembly = 0.175604626709 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1964,7 +2035,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.383870968</v>
+        <v>0.3154574132492114</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -1984,6 +2055,11 @@
       <c r="G82" t="inlineStr">
         <is>
           <t>sheet rolling, aluminium</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>(35.7) kg / 113.169 kg dry assembly = 0.315457413249 kg/kg. Processing service; excluded from material mass balance. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -1994,7 +2070,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.459365591</v>
+        <v>0.377497371188223</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2014,6 +2090,11 @@
       <c r="G83" t="inlineStr">
         <is>
           <t>aluminium alloy, AlLi</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>(35.7 + 7.021) kg / 113.169 kg dry assembly = 0.377497371188 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2105,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.060139785</v>
+        <v>0.04942166140904311</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2044,6 +2125,11 @@
       <c r="G84" t="inlineStr">
         <is>
           <t>glass fibre</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>(5.593) kg / 113.169 kg dry assembly = 0.049421661409 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2140,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.049903226</v>
+        <v>0.04100946372239748</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2074,6 +2160,11 @@
       <c r="G85" t="inlineStr">
         <is>
           <t>polyurethane, flexible foam</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>(4.641) kg / 113.169 kg dry assembly = 0.0410094637224 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(inventories): remove stationary buffers from EV chargers
Remove the storage-battery input from five charger datasets across the bus, final-energy, legacy truck-component and regional truck inventories. Document the charger boundary without dedicated stationary storage.

Validated all 406 imported datasets against the originals: only five storage inputs and their charger comments changed. Workbook formulas, cached values and unrelated archive members are preserved.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-truck-legacy-components.xlsx
+++ b/premise/data/additional_inventories/lci-truck-legacy-components.xlsx
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retained legacy truck component, ecoinvent 3.7 import basis; not regenerated by the current vehicle model. </t>
+          <t>Retained legacy truck component, ecoinvent 3.7 import basis; not regenerated by the current vehicle model.  Stationary buffer battery excluded: this inventory represents charging equipment without dedicated stationary storage.</t>
         </is>
       </c>
     </row>
@@ -4325,11 +4325,11 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Storage battery</t>
+          <t>Charger</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>1</v>
+        <v>4.3</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -4348,18 +4348,18 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Storage battery</t>
+          <t>Charger</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Charger</t>
+          <t>EV charger, level 3, plugin, 200 kW</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>4.3</v>
+        <v>1</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
@@ -4373,19 +4373,19 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>technosphere</t>
+          <t>production</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Charger</t>
+          <t>EV charger, level 3, plugin, 200 kW</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>EV charger, level 3, plugin, 200 kW</t>
+          <t>Charging stand</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -4403,40 +4403,10 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>production</t>
+          <t>technosphere</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
-        <is>
-          <t>EV charger, level 3, plugin, 200 kW</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>Charging stand</t>
-        </is>
-      </c>
-      <c r="B212" t="n">
-        <v>1</v>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>RER</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="F212" t="inlineStr">
-        <is>
-          <t>technosphere</t>
-        </is>
-      </c>
-      <c r="G212" t="inlineStr">
         <is>
           <t>Charging stand</t>
         </is>

</xml_diff>